<commit_message>
feat: route analysis xlsm with folder/alias parsing and full test suite
- FirewallRouteAnalysis.bas: zone-graph BFS route analysis (적용대상방화벽 경로)
- CIDR/list zone resolution, longest-prefix matching
- folder-name parsing (정보보호센터_1234 -> team/doc_no) + recursive subfolder scan
- user-defined header aliases via settings header_alias
- request xlsx parsing verification (varied layouts)
- Linux xlsm builder (pyOpenVBA + openpyxl), no Excel/PowerShell needed
- 50 passing tests (route oracle + parsing + xlsm structure)
</commit_message>
<xml_diff>
--- a/firewall-policy-automation.xlsx
+++ b/firewall-policy-automation.xlsx
@@ -10,15 +10,17 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="requests" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="firewalls" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settings" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="sample-request-format" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="usage" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="processing_log" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="sample-request-format" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="usage" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'requests'!$A$1:$N$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'requests'!$A$1:$Q$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'firewalls'!$A$1:$B$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'settings'!$A$1:$B$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'sample-request-format'!$A$1:$M$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'usage'!$A$1:$B$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'processing_log'!$A$1:$E$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'sample-request-format'!$A$1:$M$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'usage'!$A$1:$B$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -37,7 +39,6 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
     </font>
   </fonts>
   <fills count="3">
@@ -49,11 +50,11 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F4E78"/>
+        <fgColor rgb="00D9EAF7"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -61,31 +62,17 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="00D9E2F3"/>
-      </left>
-      <right style="thin">
-        <color rgb="00D9E2F3"/>
-      </right>
-      <top style="thin">
-        <color rgb="00D9E2F3"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00D9E2F3"/>
-      </bottom>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -452,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N1"/>
+  <dimension ref="A1:Q1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -469,6 +456,9 @@
     <col width="12" customWidth="1" min="12" max="12"/>
     <col width="12" customWidth="1" min="13" max="13"/>
     <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="19" customWidth="1" min="15" max="15"/>
+    <col width="20" customWidth="1" min="16" max="16"/>
+    <col width="15" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -542,9 +532,24 @@
           <t>비고</t>
         </is>
       </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>validation_status</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>validation_message</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>match_details</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N1"/>
+  <autoFilter ref="A1:Q1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -575,36 +580,36 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>FW-INTERNAL-01</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>10.10.0.0/16;172.16.1.0/24</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>FW-DMZ-01</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>10.20.0.0/16;172.16.20.0/24</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>FW-SERVER-01</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>10.30.0.0/16;172.16.30.0/24</t>
         </is>
@@ -625,8 +630,8 @@
   <dimension ref="A1:B3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -642,20 +647,20 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>request_folder</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr"/>
+      <c r="B2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>parse_targets</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>출발지IP;목적지IP</t>
         </is>
@@ -668,6 +673,55 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>processed_at</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>source_file</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>merged_rows</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>message</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:E1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -692,7 +746,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr"/>
+      <c r="A1" s="1" t="n"/>
       <c r="B1" s="1" t="inlineStr">
         <is>
           <t>No</t>
@@ -755,61 +809,60 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr"/>
-      <c r="B2" s="2" t="n">
+      <c r="B2" t="n">
         <v>1</v>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>10.10.10.0/24</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>업무PC</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>172.16.1.10</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>업무시스템</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>TCP</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>443</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>IN</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>HTTPS 업무 연동</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>2026-01-01</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>2026-12-31</t>
         </is>
       </c>
-      <c r="M2" s="2" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>정기 신청</t>
         </is>
@@ -821,7 +874,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -831,7 +884,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="90" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -847,64 +900,62 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
+      <c r="A2" t="n">
         <v>1</v>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Open this workbook and Save As firewall-policy-automation.xlsm if you need macros.</t>
+          <t>Save this workbook as .xlsm in Excel.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="n">
+      <c r="A3" t="n">
         <v>2</v>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Set settings!B2 to the request folder path, or run SelectRequestFolder after importing the macro.</t>
+          <t>Import vba/FirewallPolicyAutomation.bas into the VBA editor.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="n">
+      <c r="A4" t="n">
         <v>3</v>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Register firewall ranges in the firewalls sheet.</t>
+          <t>Run SetupFirewallAutomationWorkbook once to refresh sheets and headers.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="n">
+      <c r="A5" t="n">
         <v>4</v>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Put request Excel files in the request folder.</t>
+          <t>Fill firewalls!A:B with firewall_name and cidr_list.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="n">
+      <c r="A6" t="n">
         <v>5</v>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Run MergeFirewallRequestFolder after macro import.</t>
+          <t>Set settings!B2 request_folder or run SelectRequestFolder.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
+      <c r="A7" t="n">
+        <v>6</v>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>This workbook is preconfigured, but real embedded VBA macro generation requires Excel/vbaProject.bin.</t>
+          <t>Run MergeFirewallRequestFolder. Review requests validation columns and processing_log.</t>
         </is>
       </c>
     </row>

</xml_diff>